<commit_message>
Daily slate 2026-06-09 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-06-07.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-06-07.xlsx
@@ -471,16 +471,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="E2" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F2" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G2" t="n">
-        <v>51.9</v>
+        <v>52.4</v>
       </c>
     </row>
     <row r="3">
@@ -500,16 +500,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="E3" t="n">
         <v>85</v>
       </c>
       <c r="F3" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="G3" t="n">
-        <v>55.2</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="4">
@@ -529,16 +529,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E4" t="n">
         <v>25</v>
       </c>
       <c r="F4" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G4" t="n">
-        <v>42.4</v>
+        <v>41.7</v>
       </c>
     </row>
     <row r="5">
@@ -558,16 +558,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="E5" t="n">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="F5" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G5" t="n">
-        <v>52.7</v>
+        <v>53.8</v>
       </c>
     </row>
     <row r="6">
@@ -587,16 +587,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E6" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F6" t="n">
         <v>41</v>
       </c>
       <c r="G6" t="n">
-        <v>43.1</v>
+        <v>43.8</v>
       </c>
     </row>
     <row r="7">
@@ -616,16 +616,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F7" t="n">
         <v>9</v>
       </c>
       <c r="G7" t="n">
-        <v>43.8</v>
+        <v>47.1</v>
       </c>
     </row>
     <row r="8">
@@ -732,16 +732,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1073</v>
+        <v>1105</v>
       </c>
       <c r="E11" t="n">
-        <v>635</v>
+        <v>649</v>
       </c>
       <c r="F11" t="n">
-        <v>438</v>
+        <v>456</v>
       </c>
       <c r="G11" t="n">
-        <v>59.2</v>
+        <v>58.7</v>
       </c>
     </row>
     <row r="12">
@@ -761,16 +761,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="E12" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F12" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="G12" t="n">
-        <v>62.9</v>
+        <v>62.1</v>
       </c>
     </row>
     <row r="13">
@@ -819,16 +819,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>326</v>
+        <v>338</v>
       </c>
       <c r="E14" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F14" t="n">
-        <v>248</v>
+        <v>259</v>
       </c>
       <c r="G14" t="n">
-        <v>23.9</v>
+        <v>23.4</v>
       </c>
     </row>
     <row r="15">
@@ -848,16 +848,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>416</v>
+        <v>432</v>
       </c>
       <c r="E15" t="n">
         <v>88</v>
       </c>
       <c r="F15" t="n">
-        <v>328</v>
+        <v>344</v>
       </c>
       <c r="G15" t="n">
-        <v>21.2</v>
+        <v>20.4</v>
       </c>
     </row>
     <row r="16">
@@ -906,16 +906,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>4192</v>
+        <v>4335</v>
       </c>
       <c r="E17" t="n">
-        <v>867</v>
+        <v>879</v>
       </c>
       <c r="F17" t="n">
-        <v>3325</v>
+        <v>3456</v>
       </c>
       <c r="G17" t="n">
-        <v>20.7</v>
+        <v>20.3</v>
       </c>
     </row>
   </sheetData>
@@ -1489,16 +1489,16 @@
         <v>129</v>
       </c>
       <c r="D7" t="n">
-        <v>59.2</v>
+        <v>58.7</v>
       </c>
       <c r="E7" t="n">
-        <v>1073</v>
+        <v>1105</v>
       </c>
       <c r="F7" t="n">
-        <v>62.9</v>
+        <v>62.1</v>
       </c>
       <c r="G7" t="n">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="H7" t="n">
         <v>64.59999999999999</v>
@@ -1507,16 +1507,16 @@
         <v>48</v>
       </c>
       <c r="J7" t="n">
-        <v>23.9</v>
+        <v>23.4</v>
       </c>
       <c r="K7" t="n">
-        <v>326</v>
+        <v>338</v>
       </c>
       <c r="L7" t="n">
-        <v>21.2</v>
+        <v>20.4</v>
       </c>
       <c r="M7" t="n">
-        <v>416</v>
+        <v>432</v>
       </c>
       <c r="N7" t="n">
         <v>26.2</v>
@@ -1525,28 +1525,28 @@
         <v>187</v>
       </c>
       <c r="P7" t="n">
-        <v>20.7</v>
+        <v>20.3</v>
       </c>
       <c r="Q7" t="n">
-        <v>4192</v>
+        <v>4335</v>
       </c>
       <c r="R7" t="n">
-        <v>51.9</v>
+        <v>52.4</v>
       </c>
       <c r="S7" t="n">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="T7" t="n">
-        <v>42.4</v>
+        <v>41.7</v>
       </c>
       <c r="U7" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="V7" t="n">
-        <v>43.1</v>
+        <v>43.8</v>
       </c>
       <c r="W7" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="X7" t="n">
         <v>37.7</v>
@@ -1555,22 +1555,22 @@
         <v>138</v>
       </c>
       <c r="Z7" t="n">
-        <v>55.2</v>
+        <v>54.5</v>
       </c>
       <c r="AA7" t="n">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="AB7" t="n">
-        <v>52.7</v>
+        <v>53.8</v>
       </c>
       <c r="AC7" t="n">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="AD7" t="n">
-        <v>43.8</v>
+        <v>47.1</v>
       </c>
       <c r="AE7" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="AF7" t="n">
         <v>100</v>

</xml_diff>